<commit_message>
docs: add OBE curriculum implementation documentation and structural matrices for SISTEKIN 2026
</commit_message>
<xml_diff>
--- a/KURIKULUM2026_ZCODE/Implementasi_Modul_OBE_SISTEKIN2026.xlsx
+++ b/KURIKULUM2026_ZCODE/Implementasi_Modul_OBE_SISTEKIN2026.xlsx
@@ -5699,7 +5699,7 @@
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="57.00000000000001" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
@@ -5866,7 +5866,7 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Digital Governance Analyst (Analis Tata Kelola TI)</t>
+          <t>Digital System &amp; Technology Governance Analyst (Analis Tata Kelola Sistem &amp; TI)</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
@@ -11292,7 +11292,7 @@
     <col width="11.9" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="35" customWidth="1" min="5" max="5"/>
-    <col width="49.3" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -11450,7 +11450,7 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>22</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
@@ -11465,7 +11465,7 @@
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>19 SKS (2 MK 0-SKS MKWU kebijakan UWG)</t>
+          <t>22 SKS (8 MK ber-SKS + 2 MK @ 0 SKS kebijakan UWG)</t>
         </is>
       </c>
     </row>
@@ -11593,7 +11593,7 @@
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>Single track TA; syarat lulus = 144 SKS</t>
+          <t>Single track TA; syarat kelulusan minimal = 144 SKS</t>
         </is>
       </c>
     </row>
@@ -11610,18 +11610,18 @@
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>131</t>
+          <t>154</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>(Wajib ditempuh) + 9 MK Pilihan Peminatan (27 SKS, Sem 5-7) = 61 MK / 170 SKS</t>
+          <t>49 MK Wajib (130 SKS) + 8 MK Pilihan Peminatan (24 SKS, Sem 5-7) = 57 MK / 154 SKS Paket Terjadwal</t>
         </is>
       </c>
       <c r="E13" s="10" t="inlineStr"/>
       <c r="F13" s="10" t="inlineStr">
         <is>
-          <t>Portofolio 170 SKS; syarat lulus 144 SKS</t>
+          <t>Portofolio Ditawarkan: 67 MK / 184 SKS; Syarat Lulus: Minimal 144 SKS</t>
         </is>
       </c>
     </row>

</xml_diff>